<commit_message>
docs: close out D001 — log, calendar, and state pointer [D001]
Records D001's run log, marks its BUILD_CALENDAR.md row Done, syncs the
xlsx dashboard, and advances BUILD_STATE.md's current-card pointer to D002.
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1497,11 +1497,15 @@
       </c>
       <c r="J5" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K5" s="43" t="n"/>
-      <c r="L5" s="43" t="n"/>
+      <c r="L5" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D001.md)</t>
+        </is>
+      </c>
       <c r="M5" s="44" t="inlineStr">
         <is>
           <t>D001</t>

</xml_diff>

<commit_message>
feat(config): add regression test for shared strict tsconfig [D002]
D001 already put strict:true into packages/config/tsconfig.base.json
and wired per-package typecheck scripts, so pnpm typecheck was already
green — but nothing regression-tested that guarantee. Adds a Vitest
suite that type-checks fixtures against the real base config, proving
noImplicitAny, strictNullChecks, and noUncheckedIndexedAccess actually
reject unsafe code (verified by temporarily disabling strict and
confirming the test fails, then restoring it).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1565,11 +1565,15 @@
       </c>
       <c r="J6" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K6" s="43" t="n"/>
-      <c r="L6" s="43" t="n"/>
+      <c r="L6" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D002.md)</t>
+        </is>
+      </c>
       <c r="M6" s="44" t="inlineStr">
         <is>
           <t>D002</t>

</xml_diff>

<commit_message>
feat(lint): add ESLint + Prettier with custom raw-SQL ban [D003]
New @smb-os/eslint-config shares a flat ESLint 10 config across every
package, including a custom local/no-raw-sql rule that errors on raw SQL
literals, sql`` tagged templates, and .query()/.execute() calls anywhere
outside packages/db — the one package responsible for dialect handling
and tenant scoping. Verified against a deliberate violation in apps/api
(reverted after confirming lint failed) and against packages/db's
allowRawSql escape hatch (confirmed clean).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1633,11 +1633,15 @@
       </c>
       <c r="J7" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K7" s="43" t="n"/>
-      <c r="L7" s="43" t="n"/>
+      <c r="L7" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D003.md)</t>
+        </is>
+      </c>
       <c r="M7" s="44" t="inlineStr">
         <is>
           <t>D003</t>

</xml_diff>

<commit_message>
docs: close out D004 — log, calendar, and state pointer [D004]
Records D004 (test harness / Vitest coverage thresholds) as Done in
docs/logs/D004.md and docs/BUILD_CALENDAR.md, advances BUILD_STATE.md's
current-card pointer to D005, and syncs the human-facing xlsx dashboard.
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1701,11 +1701,15 @@
       </c>
       <c r="J8" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K8" s="43" t="n"/>
-      <c r="L8" s="43" t="n"/>
+      <c r="L8" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D004.md)</t>
+        </is>
+      </c>
       <c r="M8" s="44" t="inlineStr">
         <is>
           <t>D004</t>

</xml_diff>

<commit_message>
feat(ci): add CI pipeline skeleton [D005]
Add .github/workflows/ci.yml running frozen-lockfile install, lint,
typecheck, test, and test:isolation on every PR and push to main.
Test-first via packages/config/test/ci-workflow.test.ts, which asserts
the workflow triggers on pull_request, installs with
--frozen-lockfile, and runs the gate steps in dependency order.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1769,11 +1769,15 @@
       </c>
       <c r="J9" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K9" s="43" t="n"/>
-      <c r="L9" s="43" t="n"/>
+      <c r="L9" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D005.md)</t>
+        </is>
+      </c>
       <c r="M9" s="44" t="inlineStr">
         <is>
           <t>D005</t>

</xml_diff>

<commit_message>
feat(security): add gitleaks secret scanning to pre-commit and CI [D006]
Wires gitleaks into a local pre-commit hook (auto-installed via a new
package.json prepare script) and into CI (install step + repo-wide
detect scan with fetch-depth: 0), test-first via a vitest spec that
plants a fake secret and asserts detection.
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1837,11 +1837,15 @@
       </c>
       <c r="J10" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K10" s="43" t="n"/>
-      <c r="L10" s="43" t="n"/>
+      <c r="L10" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D006.md)</t>
+        </is>
+      </c>
       <c r="M10" s="44" t="inlineStr">
         <is>
           <t>D006</t>

</xml_diff>

<commit_message>
docs: record D007 commit hash in log [D007]
Close out D007 — dependency scanning and SBOM: BUILD_CALENDAR/xlsx
status Done, BUILD_STATE current-card pointer moved to D008.
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1905,11 +1905,15 @@
       </c>
       <c r="J11" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K11" s="43" t="n"/>
-      <c r="L11" s="43" t="n"/>
+      <c r="L11" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D007.md)</t>
+        </is>
+      </c>
       <c r="M11" s="44" t="inlineStr">
         <is>
           <t>D007</t>

</xml_diff>

<commit_message>
feat(security): add semgrep SAST scanning to CI [D008]
Wires `semgrep scan --config p/security-audit --error` into CI after
pnpm audit and before lint/typecheck/test, so a high/critical finding
fails the build before any application code exists to accumulate one.
Test-first via packages/config/test/sast.test.ts against a real
command-injection fixture and a clean-fixture control.
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -1973,11 +1973,15 @@
       </c>
       <c r="J12" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K12" s="43" t="n"/>
-      <c r="L12" s="43" t="n"/>
+      <c r="L12" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D008.md)</t>
+        </is>
+      </c>
       <c r="M12" s="44" t="inlineStr">
         <is>
           <t>D008</t>

</xml_diff>

<commit_message>
feat(auth): native AuthProvider — Argon2id, sessions, rate limiting [D010]
Implements the AuthProvider interface (packages/domain, no I/O) and a
NativeAuthProvider (apps/api) per ADR-002: Argon2id password hashing,
opaque revocable session cookies (httpOnly/Secure/SameSite=Strict),
hashed single-use password-reset tokens, per-IP and per-account rate
limiting on login/reset-request, progressive account lockout, and an
Origin-header CSRF check. Persistence is in-memory behind repository
interfaces pending D013-D015's real Drizzle/DB wiring (Phase 1).

Carried, not Done: TOTP MFA for OWNER/ADMIN (ADR-002 requirement) is
not yet implemented. See docs/logs/D010.md for the full gap analysis.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -2041,11 +2041,15 @@
       </c>
       <c r="J13" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K13" s="43" t="n"/>
-      <c r="L13" s="43" t="n"/>
+      <c r="L13" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D009.md)</t>
+        </is>
+      </c>
       <c r="M13" s="44" t="inlineStr">
         <is>
           <t>D009</t>
@@ -2105,13 +2109,13 @@
       </c>
       <c r="J14" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Carried</t>
         </is>
       </c>
       <c r="K14" s="43" t="n"/>
       <c r="L14" s="43" t="inlineStr">
         <is>
-          <t>Revised per ADR-002 (2026-09-07): was 'Identity provider spike / OIDC PKCE'. Founder decision: native auth now, Auth0-ready interface, Auth0 wired in later.</t>
+          <t>[log](docs/logs/D010.md)</t>
         </is>
       </c>
       <c r="M14" s="44" t="inlineStr">

</xml_diff>

<commit_message>
docs: close out D011, advance current-card pointer to D012 [D011]
Marks D011 Done in BUILD_CALENDAR.md and the xlsx dashboard, writes
docs/logs/D011.md with the acceptance-criteria and security-check
answers, and moves BUILD_STATE.md's current-card pointer to D012
(threat model, IR plan, subprocessors — Gate G0).
</commit_message>
<xml_diff>
--- a/docs/implementation_calendar/build_calendar.xlsx
+++ b/docs/implementation_calendar/build_calendar.xlsx
@@ -2041,11 +2041,15 @@
       </c>
       <c r="J13" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K13" s="43" t="n"/>
-      <c r="L13" s="43" t="n"/>
+      <c r="L13" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D009.md)</t>
+        </is>
+      </c>
       <c r="M13" s="44" t="inlineStr">
         <is>
           <t>D009</t>
@@ -2105,13 +2109,13 @@
       </c>
       <c r="J14" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K14" s="43" t="n"/>
       <c r="L14" s="43" t="inlineStr">
         <is>
-          <t>Revised per ADR-002 (2026-09-07): was 'Identity provider spike / OIDC PKCE'. Founder decision: native auth now, Auth0-ready interface, Auth0 wired in later.</t>
+          <t>[log](docs/logs/D010.md)</t>
         </is>
       </c>
       <c r="M14" s="44" t="inlineStr">
@@ -2173,11 +2177,15 @@
       </c>
       <c r="J15" s="43" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K15" s="43" t="n"/>
-      <c r="L15" s="43" t="n"/>
+      <c r="L15" s="43" t="inlineStr">
+        <is>
+          <t>[log](docs/logs/D011.md)</t>
+        </is>
+      </c>
       <c r="M15" s="44" t="inlineStr">
         <is>
           <t>D011</t>

</xml_diff>